<commit_message>
feat: GPS prompt on meals+restaurants, best-match default, tappable restaurant tag
</commit_message>
<xml_diff>
--- a/Stride_Work_Log.xlsx
+++ b/Stride_Work_Log.xlsx
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1644,13 +1644,334 @@
         </is>
       </c>
     </row>
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="9" t="inlineStr">
+        <is>
+          <t>DATABASE SCHEMA DECISIONS — 2026-05-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="32" customHeight="1">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Schema</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>Single meals table, nullable restaurant_id. Per-serving macros only (compute per-100g). Boolean diet tag columns. Three-state allergens (null/true/false). Price range for generic dishes.</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>Full schema defined in DATABASE_SCHEMA.md</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>✅ Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="32" customHeight="1">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Schema</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>Dedup: canonical_name UNIQUE + fuzzy match on submit + duplicate rows kept with self-FK (never delete — protects user logs)</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>Prevents MyFitnessPal naming problem</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>✅ Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="32" customHeight="1">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Schema</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>Community stats: separate pre-aggregated table, recomputed on feedback approval. Show only when count&gt;=3. Range display when std_dev&gt;20%.</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>Fast queries, reliable community data display</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>✅ Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="32" customHeight="1">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>DATABASE_SCHEMA.md created in OneDrive Fitness App root. Full SQL schema, design decisions, sgFoodDb mapping, display rules.</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>Single source of truth for schema</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>✅ Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="32" customHeight="1">
+      <c r="A50" s="12" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="B50" s="12" t="inlineStr">
+        <is>
+          <t>Implementation</t>
+        </is>
+      </c>
+      <c r="C50" s="13" t="inlineStr">
+        <is>
+          <t>Implement allergens field in sgFoodDb.ts TypeScript schema + populate from official SG PDFs for top chains</t>
+        </is>
+      </c>
+      <c r="D50" s="13" t="inlineStr">
+        <is>
+          <t>Allergen data live for Stride Approved meals</t>
+        </is>
+      </c>
+      <c r="E50" s="12" t="inlineStr">
+        <is>
+          <t>⏳ Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="18" customHeight="1">
+      <c r="A51" s="9" t="inlineStr">
+        <is>
+          <t>INFRASTRUCTURE DECISION — 2026-05-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="32" customHeight="1">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>Stay on Firebase/Firestore. Four collections: /restaurants, /meals, /meal_feedback, /meal_community_stats. sgFoodDb.ts stays as client-side search layer.</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>No second backend. Search stays fast and offline. Community stats via Cloud Function.</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>✅ Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="18" customHeight="1">
+      <c r="A53" s="9" t="inlineStr">
+        <is>
+          <t>ALLERGEN SCHEMA &amp; MVP DECISION — 2026-05-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="28" customHeight="1">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Schema</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>SGAllergens interface + allergens?: SGAllergens field added to SGMenuItem. Three-state: true=contains, false=verified free, null=unknown.</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>Schema ready for data population</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="28" customHeight="1">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>McDonald's 11 items populated with allergen data. Some fields still null (McSpicy eggs, Fries shared fryer, Cone mix) — need official PDF verification.</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>First real allergen data in the system</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="28" customHeight="1">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>Allergen data logged in schema but NOT displayed in app UI for MVP. Too dangerous to show partial/unverified allergen claims. Phase 2: verify nulls from official SG PDFs, then build UI display.</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>Safety over completeness — log now, display later</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>✅ Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="28" customHeight="1">
+      <c r="A57" s="12" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="B57" s="12" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="C57" s="13" t="inlineStr">
+        <is>
+          <t>KFC, Subway, Burger King, and all other outlets: allergen fields not yet populated. Dean to populate from official SG allergen PDFs/guides.</t>
+        </is>
+      </c>
+      <c r="D57" s="13" t="inlineStr">
+        <is>
+          <t>Full allergen coverage across all outlets</t>
+        </is>
+      </c>
+      <c r="E57" s="12" t="inlineStr">
+        <is>
+          <t>⏳ Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="28" customHeight="1">
+      <c r="A58" s="12" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="B58" s="12" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="C58" s="13" t="inlineStr">
+        <is>
+          <t>Build allergen display layer in Eat tab and Log tab. Show badges only for source='official_sg'|'hpb'. Always include disclaimer.</t>
+        </is>
+      </c>
+      <c r="D58" s="13" t="inlineStr">
+        <is>
+          <t>Allergen filtering live for users</t>
+        </is>
+      </c>
+      <c r="E58" s="12" t="inlineStr">
+        <is>
+          <t>⏳ Pending</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="9">
     <mergeCell ref="A39:E39"/>
+    <mergeCell ref="A53:E53"/>
     <mergeCell ref="A12:E12"/>
     <mergeCell ref="A35:E35"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A51:E51"/>
+    <mergeCell ref="A45:E45"/>
     <mergeCell ref="A27:E27"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1663,7 +1984,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2548,14 +2869,550 @@
         </is>
       </c>
     </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="9" t="inlineStr">
+        <is>
+          <t>DATABASE SCHEMA DECISIONS — 2026-05-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="58" customHeight="1">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Schema: Meal Table Structure</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Single meals table with nullable restaurant_id for all food items (restaurant menu items AND generic hawker/HPB dishes)</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>Both types share 90% of fields. Two separate tables would duplicate search logic and require UNION queries. restaurant_id=NULL cleanly distinguishes generic dishes from outlet-specific items.</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>Two separate tables: restaurant_meals + generic_meals (JOIN complexity, duplicate search logic)</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>✅ Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="58" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Schema: Macros Storage</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Store macros per serving + serving_size_g only. Never store per-100g — always compute: macro_per_100g = (macro / serving_size_g) × 100</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>Storing both creates a sync problem: if serving_size_g is corrected, pre-computed per-100g values become stale. Single source of truth is the per-serving values.</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>Store both per-serving and per-100g (sync risk), Store only per-100g (loses serving context)</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>✅ Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="58" customHeight="1">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Schema: Diet Tag Columns</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Core diet tags as boolean columns (is_halal, is_vegetarian, is_vegan, is_keto, is_gluten_free, is_high_protein). Extras in diet_tags_extra TEXT[].</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>Boolean columns are indexed and fast: WHERE is_halal=true AND is_vegan=true uses B-tree index. Array @&gt; operator requires GIN index and is slower. is_high_protein is computed (protein_g &gt;= 25) but stored as column so it is indexed.</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>Single TEXT[] column for all tags (slow array queries), JSON column (no indexing), Bitmask integer (unreadable)</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>✅ Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="58" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Schema: Allergen Three-State</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Allergen columns are BOOLEAN? (nullable): NULL=unknown (show nothing), TRUE=contains (show warning), FALSE=verified free (show with disclaimer). Only populated from official_sg or hpb sources.</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>Wrong allergen data causes physical harm. NULL forces the app to show nothing rather than a wrong claim. False-negative allergen labelling (saying nut-free when it is not) could cause anaphylaxis. Showing nothing is always safer than showing unverified absence claims.</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>Boolean only true/false (no unknown state), Text array of allergens present (no verified-free state), Skip allergens entirely</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>✅ Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="58" customHeight="1">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Schema: Price Fields</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Restaurant items: single price_sgd. Generic dishes: price_min_sgd, price_max_sgd, price_typical_sgd range. Both types have all four columns; unused ones are NULL.</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>Chicken rice is $3.50 at a hawker and $12 at a hotel. A single price field is misleading for generic dishes. A range with a typical value gives users useful context. Restaurant items always have a fixed price from the official menu.</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>Single price field for all (misleading for generic dishes), Always store ranges (unnecessary for fixed-price restaurant items)</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>✅ Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="58" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Schema: Deduplication</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>canonical_name (UNIQUE) + aliases[] + status (active/duplicate/archived) + canonical_meal_id self-FK. Fuzzy match on submission: &gt;80% = block, 60-80% = warn. Duplicate rows are never deleted — they stay with status=duplicate pointing to canonical.</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>MyFitnessPal failure: unchecked community entries created thousands of near-duplicate meals. Prevention (fuzzy match on submit) + cleanup (admin merge queue) is the solution. Keeping duplicate rows protects existing user food logs that reference them.</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>Delete duplicates (breaks user food logs), No deduplication (MyFitnessPal problem), Manual only with no system enforcement</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>✅ Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="58" customHeight="1">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Schema: Community Stats Separation</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>meal_community_stats is a separate table, recomputed when feedback is approved. Never aggregate at query time. Show community data only when feedback_count &gt;= 3. Show range (not average) when std_dev_calories &gt; 20% of avg.</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>Recomputing averages across thousands of feedback rows on every search query is too slow. Pre-aggregated stats give instant reads. std_dev is a reliability signal: high variance means the community does not agree on the macros — show a range instead of a misleading precise number.</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>Compute averages on every query (too slow at scale), Show all feedback regardless of count (n=1 is unreliable)</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>✅ Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="58" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Schema: Confidence Tier Display</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Three tiers: stride_approved (official_sg/hpb + verified) shows allergens + full data. community (feedback_count&gt;=3) shows macros + Community badge, no allergens. stride_estimate (usda/extracted) shows macros + Estimate badge, no allergens.</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>Users need to know how much to trust the data they see. Allergen data is only shown when we have official verification — community and estimated items never show allergen claims regardless of confidence.</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>No confidence display (users cannot assess data quality), Single verified/unverified flag (loses source context)</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>✅ Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="9" t="inlineStr">
+        <is>
+          <t>INFRASTRUCTURE DECISION — 2026-05-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="55" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Database Platform</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Stay on Firebase / Firestore. Food database built as Firestore collections. Do NOT migrate to Supabase.</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>Already set up, already paid for, already wired to auth and user data. Choo Ming Hao's roadmap listed Supabase as an option, but splitting to two backend services adds unnecessary complexity at this stage. Firestore collections map directly to the schema we designed.</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>Supabase/PostgreSQL (clean SQL but adds second backend service, migration cost, extra complexity)</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>✅ Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="55" customHeight="1">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Firestore Collection Structure</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Four collections: /restaurants/{id}, /meals/{id}, /meal_feedback/{id}, /meal_community_stats/{mealId}. meal_community_stats uses same ID as the meal document it aggregates.</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>Direct mapping of the schema tables to Firestore collections. meal_community_stats keyed by meal ID enables single-document lookup without a query.</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>Subcollections under meals (harder to query across meals), Single flat collection (no separation of concerns)</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>✅ Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="58" customHeight="1">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Firestore: Search Strategy</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>Keep sgFoodDb.ts as the client-side search layer (fast, offline, no Firestore reads). Use Firestore for persistence, user feedback, and community stats only. Algolia can be added later if search scale demands it.</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>Firestore cannot do substring text search (no LIKE queries). sgFoodDb.ts already provides fast client-side search via searchAll(). This avoids paying for Algolia at MVP stage while keeping search fast. Firestore array-contains works for exact alias matching.</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>Algolia now (cost, complexity at MVP stage), Firestore-only search (no substring support without workarounds)</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>✅ Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="50" customHeight="1">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Firestore: Computed Fields</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>is_high_protein and confidence_tier are computed at write time and stored as explicit fields. Do not derive on read.</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>Firestore has no computed columns. Storing pre-computed values keeps reads fast and queries simple. is_high_protein = protein_g &gt;= 25, set on every meal write/update.</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>Compute on read (slower, more code), Cloud Functions for computation (over-engineered for two fields)</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>✅ Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="50" customHeight="1">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Firestore: Community Stats Update</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>meal_community_stats document updated via Cloud Function triggered on meal_feedback status change to 'approved'. Never aggregate at query time.</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>Firestore has no native aggregation. Pre-aggregated document is read in a single document fetch at query time. Cloud Function keeps it current without blocking the user-facing write.</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>Aggregate on every read (too slow at scale), Client-side aggregation (race conditions, inconsistent)</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>✅ Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="9" t="inlineStr">
+        <is>
+          <t>ALLERGEN MVP STRATEGY — 2026-05-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="60" customHeight="1">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Allergen Display — MVP Decision</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>Allergen data is logged in sgFoodDb.ts schema but NOT displayed in the app UI for MVP. Post-MVP, display only after full verification from official SG PDFs.</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>Incomplete allergen data shown in the UI is more dangerous than showing none. A user with a peanut allergy who sees 'peanuts: false' on an unverified item may be seriously harmed. The right order: log everything now → verify against official SG allergen PDFs → build UI display only after verification is complete.</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>Show available allergen data now with a disclaimer (still shows unverified claims), Skip allergen logging entirely (loses data we've already gathered)</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>✅ Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="55" customHeight="1">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Allergen Data — Phase Plan</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>Phase 1 (now): log allergen data as researched, null for unknowns, no UI display. Phase 2 (post-MVP): verify all null fields from official SG PDFs, build UI display for official_sg/hpb items only, add disclaimer on all allergen info shown.</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>Separating logging from display lets us capture data progressively without creating a safety risk. McDonald's SG top items partially populated. KFC, Subway, and all other outlets still need population. UI layer not yet built.</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>Build display and data together (blocks on full verification), Log and display simultaneously (safety risk with partial data)</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>✅ Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="55" customHeight="1">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Allergen Schema Implementation</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>SGAllergens interface added to sgFoodDb.ts. allergens?: SGAllergens field added to SGMenuItem. McDonald's 11 core items populated with allergen data (mix of true/false/null). MVP notice comment added at top of interface.</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>Schema is in place and typed correctly. null fields on McDonald's items (McSpicy coating eggs, fries shared fryer, Cone soft serve mix) need verification from mcdonalds.com.sg allergen PDF before being set to true/false.</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>No schema yet (delays future implementation), Full population before schema (puts content before structure)</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="9">
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="A42:F42"/>
     <mergeCell ref="A23:F23"/>
     <mergeCell ref="A27:F27"/>
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="A17:F17"/>
     <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A48:F48"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>